<commit_message>
Data sync: 70 words · 200 phrases · 0 new images
</commit_message>
<xml_diff>
--- a/update_data_folder/Daily_Expressions.xlsx
+++ b/update_data_folder/Daily_Expressions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miaofang/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miaofang/Desktop/VocabWorkspace/update_data_folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A285FF-BD39-5941-BC53-9CD86A0B0042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C48308-E997-9041-91A1-57E9E87672F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="968">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1205" uniqueCount="968">
   <si>
     <t>Word / Expression</t>
   </si>
@@ -6712,6 +6712,9 @@
       <c r="B170" s="1" t="s">
         <v>829</v>
       </c>
+      <c r="C170" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="D170" s="1" t="s">
         <v>830</v>
       </c>

</xml_diff>